<commit_message>
version 0.6.0 custom query and append specified
</commit_message>
<xml_diff>
--- a/docs/observations-summary.xlsx
+++ b/docs/observations-summary.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="27">
   <si>
     <t>Profile</t>
   </si>
@@ -47,10 +47,10 @@
     <t>Method</t>
   </si>
   <si>
-    <t>dme-left-eye-observation</t>
-  </si>
-  <si>
-    <t>Diabetic Macular Edema Left Eye Observation</t>
+    <t>retina-diabetic-macular-edema-finding</t>
+  </si>
+  <si>
+    <t>Retina Diabetic Macular Edema Finding</t>
   </si>
   <si>
     <t/>
@@ -68,58 +68,31 @@
     <t>optional</t>
   </si>
   <si>
-    <t>SNOMED CT#58443009</t>
-  </si>
-  <si>
-    <t>dme-right-eye-observation</t>
-  </si>
-  <si>
-    <t>Diabetic Macular Edema Right Eye Observation</t>
-  </si>
-  <si>
-    <t>SNOMED CT#5597008</t>
-  </si>
-  <si>
-    <t>dr-left-eye-observation</t>
-  </si>
-  <si>
-    <t>Diabetic Retinopathy Left Eye Observation</t>
+    <t>retina-diabetic-retinopathy-finding</t>
+  </si>
+  <si>
+    <t>Retina Diabetic Retinopathy Finding</t>
   </si>
   <si>
     <t>SNOMED CT#4855003</t>
   </si>
   <si>
-    <t>dr-right-eye-observation</t>
-  </si>
-  <si>
-    <t>Diabetic Retinopathy Right Eye Observation</t>
-  </si>
-  <si>
-    <t>fundus-foto-observation</t>
-  </si>
-  <si>
-    <t>Fundus Photography Observation</t>
-  </si>
-  <si>
-    <t>no-kodeverk-7275#CKDP10</t>
-  </si>
-  <si>
-    <t>hba1c-observation</t>
-  </si>
-  <si>
-    <t>HbA1c Observation</t>
+    <t>retina-hba1c-observation</t>
+  </si>
+  <si>
+    <t>Retina HbA1c Observation</t>
   </si>
   <si>
     <t>SNOMED CT#167491000202108</t>
   </si>
   <si>
-    <t>oct-observation</t>
-  </si>
-  <si>
-    <t>OCT Observation</t>
-  </si>
-  <si>
-    <t>no-kodeverk-7275#CKFX16</t>
+    <t>retina-image-quality-asessment</t>
+  </si>
+  <si>
+    <t>Retina Image Quality Assessment</t>
+  </si>
+  <si>
+    <t>SNOMED CT#133887000</t>
   </si>
 </sst>
 </file>
@@ -253,7 +226,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -320,7 +293,7 @@
         <v>17</v>
       </c>
       <c r="J2" t="s" s="2">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="K2" t="s" s="2">
         <v>13</v>
@@ -328,19 +301,19 @@
     </row>
     <row r="3">
       <c r="A3" t="s" s="2">
+        <v>18</v>
+      </c>
+      <c r="B3" t="s" s="2">
         <v>19</v>
       </c>
-      <c r="B3" t="s" s="2">
+      <c r="C3" t="s" s="2">
+        <v>13</v>
+      </c>
+      <c r="D3" t="s" s="2">
+        <v>13</v>
+      </c>
+      <c r="E3" t="s" s="2">
         <v>20</v>
-      </c>
-      <c r="C3" t="s" s="2">
-        <v>13</v>
-      </c>
-      <c r="D3" t="s" s="2">
-        <v>13</v>
-      </c>
-      <c r="E3" t="s" s="2">
-        <v>14</v>
       </c>
       <c r="F3" t="s" s="2">
         <v>13</v>
@@ -355,7 +328,7 @@
         <v>17</v>
       </c>
       <c r="J3" t="s" s="2">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="K3" t="s" s="2">
         <v>13</v>
@@ -363,19 +336,19 @@
     </row>
     <row r="4">
       <c r="A4" t="s" s="2">
+        <v>21</v>
+      </c>
+      <c r="B4" t="s" s="2">
         <v>22</v>
       </c>
-      <c r="B4" t="s" s="2">
+      <c r="C4" t="s" s="2">
+        <v>13</v>
+      </c>
+      <c r="D4" t="s" s="2">
+        <v>13</v>
+      </c>
+      <c r="E4" t="s" s="2">
         <v>23</v>
-      </c>
-      <c r="C4" t="s" s="2">
-        <v>13</v>
-      </c>
-      <c r="D4" t="s" s="2">
-        <v>13</v>
-      </c>
-      <c r="E4" t="s" s="2">
-        <v>24</v>
       </c>
       <c r="F4" t="s" s="2">
         <v>13</v>
@@ -390,7 +363,7 @@
         <v>17</v>
       </c>
       <c r="J4" t="s" s="2">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="K4" t="s" s="2">
         <v>13</v>
@@ -398,19 +371,19 @@
     </row>
     <row r="5">
       <c r="A5" t="s" s="2">
+        <v>24</v>
+      </c>
+      <c r="B5" t="s" s="2">
         <v>25</v>
       </c>
-      <c r="B5" t="s" s="2">
+      <c r="C5" t="s" s="2">
+        <v>13</v>
+      </c>
+      <c r="D5" t="s" s="2">
+        <v>13</v>
+      </c>
+      <c r="E5" t="s" s="2">
         <v>26</v>
-      </c>
-      <c r="C5" t="s" s="2">
-        <v>13</v>
-      </c>
-      <c r="D5" t="s" s="2">
-        <v>13</v>
-      </c>
-      <c r="E5" t="s" s="2">
-        <v>24</v>
       </c>
       <c r="F5" t="s" s="2">
         <v>13</v>
@@ -425,114 +398,9 @@
         <v>17</v>
       </c>
       <c r="J5" t="s" s="2">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="K5" t="s" s="2">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s" s="2">
-        <v>27</v>
-      </c>
-      <c r="B6" t="s" s="2">
-        <v>28</v>
-      </c>
-      <c r="C6" t="s" s="2">
-        <v>13</v>
-      </c>
-      <c r="D6" t="s" s="2">
-        <v>13</v>
-      </c>
-      <c r="E6" t="s" s="2">
-        <v>29</v>
-      </c>
-      <c r="F6" t="s" s="2">
-        <v>13</v>
-      </c>
-      <c r="G6" t="s" s="2">
-        <v>15</v>
-      </c>
-      <c r="H6" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="I6" t="s" s="2">
-        <v>17</v>
-      </c>
-      <c r="J6" t="s" s="2">
-        <v>13</v>
-      </c>
-      <c r="K6" t="s" s="2">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s" s="2">
-        <v>30</v>
-      </c>
-      <c r="B7" t="s" s="2">
-        <v>31</v>
-      </c>
-      <c r="C7" t="s" s="2">
-        <v>13</v>
-      </c>
-      <c r="D7" t="s" s="2">
-        <v>13</v>
-      </c>
-      <c r="E7" t="s" s="2">
-        <v>32</v>
-      </c>
-      <c r="F7" t="s" s="2">
-        <v>13</v>
-      </c>
-      <c r="G7" t="s" s="2">
-        <v>15</v>
-      </c>
-      <c r="H7" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="I7" t="s" s="2">
-        <v>17</v>
-      </c>
-      <c r="J7" t="s" s="2">
-        <v>13</v>
-      </c>
-      <c r="K7" t="s" s="2">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s" s="2">
-        <v>33</v>
-      </c>
-      <c r="B8" t="s" s="2">
-        <v>34</v>
-      </c>
-      <c r="C8" t="s" s="2">
-        <v>13</v>
-      </c>
-      <c r="D8" t="s" s="2">
-        <v>13</v>
-      </c>
-      <c r="E8" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="F8" t="s" s="2">
-        <v>13</v>
-      </c>
-      <c r="G8" t="s" s="2">
-        <v>15</v>
-      </c>
-      <c r="H8" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="I8" t="s" s="2">
-        <v>17</v>
-      </c>
-      <c r="J8" t="s" s="2">
-        <v>13</v>
-      </c>
-      <c r="K8" t="s" s="2">
         <v>13</v>
       </c>
     </row>

</xml_diff>